<commit_message>
Update Excel and JSON data with verified live BIST prices (DSTKF 2048 TL)
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H124"/>
+  <dimension ref="A1:H135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -531,7 +531,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -763,14 +762,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>200</v>
+        <v>297</v>
       </c>
       <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] 200.00 seviyesinden alttan ekleme yapilabilir.</t>
+          <t>[Oğuz Analizi] 286₺ Astor bakılabilir, 295₺ ve 299₺ dirençleri.</t>
         </is>
       </c>
     </row>
@@ -907,7 +906,7 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>89.84999999999999</v>
+        <v>151.8</v>
       </c>
       <c r="E15" s="8" t="n">
         <v>90</v>
@@ -916,7 +915,7 @@
       <c r="G15" s="7" t="n"/>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] 90.00 ustu hareketler pozitif.</t>
+          <t>[Oğuz Analizi] 75₺'den 90₺ ve 107.60₺ seviyesine hareket.</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1084,7 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>7</v>
+        <v>6.03</v>
       </c>
       <c r="E21" s="8" t="n">
         <v>7</v>
@@ -1094,7 +1093,7 @@
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Devre kesici sonrasi 7.00 seviyesinden tepki alir.</t>
+          <t>[Oğuz Analizi] Ekos 6₺ seviyesinden bakılabilir.</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1143,9 @@
           <t>Genk/Genkm</t>
         </is>
       </c>
-      <c r="D23" s="7" t="n"/>
+      <c r="D23" s="7" t="n">
+        <v>12.18</v>
+      </c>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="7" t="n"/>
       <c r="G23" s="9" t="n">
@@ -1152,7 +1153,7 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Kisa vadede yuksek kar marji.</t>
+          <t>[Oğuz Analizi] Genkm 12.25₺ takip, yetişemeyene %4 marj.</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1202,7 @@
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>10.16</v>
+        <v>8.92</v>
       </c>
       <c r="E25" s="8" t="n">
         <v>10</v>
@@ -1212,7 +1213,7 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] 10.00 dip destegi. Tavan ile %9.91 kar verdi.</t>
+          <t>[Oğuz Analizi] Kfein 9.40₺ seviyesinden takibe alındı.</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1386,7 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>2.37</v>
+        <v>2.23</v>
       </c>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="7" t="n"/>
@@ -1394,7 +1395,7 @@
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Maliyet dusurulen noktayla %17 kar.</t>
+          <t>[Oğuz Analizi] Marmr 2.22₺ yine bakılır (%8 marj).</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1444,7 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>16.82</v>
+        <v>13.77</v>
       </c>
       <c r="E33" s="7" t="n"/>
       <c r="F33" s="7" t="n"/>
@@ -1452,7 +1453,7 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] %5 kar ile hedefe ulasti.</t>
+          <t>[Oğuz Analizi] Meysu 13.03₺ tradelik bakıyorum (%6.5 marj).</t>
         </is>
       </c>
     </row>
@@ -1500,13 +1501,15 @@
           <t>Mogan Enerji Yatirim</t>
         </is>
       </c>
-      <c r="D35" s="7" t="n"/>
+      <c r="D35" s="7" t="n">
+        <v>17.63</v>
+      </c>
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="7" t="n"/>
       <c r="G35" s="7" t="n"/>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Genel takip listesinde.</t>
+          <t>[Oğuz Analizi] Mogan 12.75₺ buradan pozisyon açıyor (%60 prim).</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1558,7 @@
         </is>
       </c>
       <c r="D37" s="8" t="n">
-        <v>147</v>
+        <v>139.3</v>
       </c>
       <c r="E37" s="7" t="n"/>
       <c r="F37" s="7" t="n"/>
@@ -1564,7 +1567,7 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Tradelik takip edildi %2 kar.</t>
+          <t>[Oğuz Analizi] Netcd 144.50₺ takibe alındı (%3.5 marj).</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1958,7 @@
         </is>
       </c>
       <c r="D51" s="8" t="n">
-        <v>83.55</v>
+        <v>81.15000000000001</v>
       </c>
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="7" t="n"/>
@@ -1964,7 +1967,7 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Tradelik takip edilebilir.</t>
+          <t>[Oğuz Analizi] Klrho 83₺ yine tradelik bakılabilir (%3.5).</t>
         </is>
       </c>
     </row>
@@ -2047,7 +2050,7 @@
         </is>
       </c>
       <c r="D54" s="5" t="n">
-        <v>29.14</v>
+        <v>28.46</v>
       </c>
       <c r="E54" s="4" t="n"/>
       <c r="F54" s="5" t="n">
@@ -2058,7 +2061,7 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Tradelik bakılabilir. 30 TL direnç.</t>
+          <t>[Oğuz Analizi] 29.20₺ üzeri takip konusu.</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2292,7 @@
         </is>
       </c>
       <c r="D62" s="5" t="n">
-        <v>38.3</v>
+        <v>39.1</v>
       </c>
       <c r="E62" s="4" t="n"/>
       <c r="F62" s="4" t="n"/>
@@ -2298,7 +2301,7 @@
       </c>
       <c r="H62" s="4" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Alınıp %5-10 marj beklenen.</t>
+          <t>[Oğuz Analizi] Bulgs 39.48₺ tradelik takip edilebilir (%3.5).</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2322,7 @@
         </is>
       </c>
       <c r="D63" s="8" t="n">
-        <v>55.55</v>
+        <v>51.65</v>
       </c>
       <c r="E63" s="7" t="n"/>
       <c r="F63" s="7" t="n"/>
@@ -2328,7 +2331,7 @@
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Yeni güncellenen hedef (%4.5).</t>
+          <t>[Oğuz Analizi] Ekinciler Demir Çelik 54.10₺ takibe alındı.</t>
         </is>
       </c>
     </row>
@@ -3950,7 +3953,9 @@
           <t>Ak Enerji Elektrik Üretim A.Ş.</t>
         </is>
       </c>
-      <c r="D118" s="4" t="n"/>
+      <c r="D118" s="4" t="n">
+        <v>10.56</v>
+      </c>
       <c r="E118" s="5" t="n">
         <v>11</v>
       </c>
@@ -3962,7 +3967,7 @@
       </c>
       <c r="H118" s="4" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Giriş: 11.00 TL | Ana Hedef: 11.51 TL (%2.5 Erken Alarm: 11.22 TL)</t>
+          <t>[Oğuz Analizi] Akenr 11₺ değerlendirip satanlar için. 10.38₺ takibi.</t>
         </is>
       </c>
     </row>
@@ -3982,7 +3987,9 @@
           <t>Yayla Enerji Üretim Turizm ve İnşaat Ticaret A.Ş.</t>
         </is>
       </c>
-      <c r="D119" s="7" t="n"/>
+      <c r="D119" s="7" t="n">
+        <v>22.98</v>
+      </c>
       <c r="E119" s="8" t="n">
         <v>23.34</v>
       </c>
@@ -3994,7 +4001,7 @@
       </c>
       <c r="H119" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Giriş: 23.34 TL | Ana Hedef: 24.06 TL (Kademeli: 23.78, 24.00) | Erken Alarm: 23.50 TL</t>
+          <t>[Oğuz Analizi] 23.10₺ ve 23.78₺ tradelik bakılabilir, 24₺ hareketi.</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4117,9 @@
           <t>Galata Wind Enerji A.Ş.</t>
         </is>
       </c>
-      <c r="D123" s="7" t="n"/>
+      <c r="D123" s="7" t="n">
+        <v>25.38</v>
+      </c>
       <c r="E123" s="8" t="n">
         <v>24.36</v>
       </c>
@@ -4122,7 +4131,7 @@
       </c>
       <c r="H123" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Giriş: 24.36 TL | Ana Hedef: 25.00 TL (Erken Alarm: 24.50 TL)</t>
+          <t>[Oğuz Analizi] Gwind 24.36₺ benzer marj beklenebilir (%7.5).</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4151,9 @@
           <t>Kron Telekomünikasyon Hizmetleri A.Ş.</t>
         </is>
       </c>
-      <c r="D124" s="4" t="n"/>
+      <c r="D124" s="4" t="n">
+        <v>24.26</v>
+      </c>
       <c r="E124" s="5" t="n">
         <v>23.8</v>
       </c>
@@ -4154,7 +4165,282 @@
       </c>
       <c r="H124" s="4" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Giriş: 23.80 TL | Ana Hedef: 24.26 TL (Erken Alarm: 24.00 TL)</t>
+          <t>[Oğuz Analizi] 22.16₺ ve 22.80₺ bakılabilir, %5 direnç bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>LILAK</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>LILAK</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Lila Kağıt Sanayi ve Ticaret</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>30.16</v>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] Lilak 30.80₺'de iyi duruyor (%2 güzel marj).</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>OBASE</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>OBASE</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Obase Bilgisayar ve Danışmanlık</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>44.44</v>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] Obase 47.98₺ seviyesinden takibe alındı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>IZMDC</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>IZMDC</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>İzmir Demir Çelik Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] Izmdc 6.156₺ buradan takip ediyorum (%110 prim).</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>AKHAN</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>AKHAN</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Akhan Un Fabrikası A.Ş.</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>40.16</v>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] 23.80₺ / 25.12₺ seviyesinden tarım emtiası takibi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>ZERGY</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>ZERGY</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Zergay Gayrimenkul Yatırım A.Ş.</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] Zergy 10.06₺ takip, 10.50₺ direnç bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>SSAAT</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>SSAAT</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Saat ve Saat Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>46.16</v>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] SSAAT 42.24₺ takip seviyesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>RUZYE</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>RUZYE</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Ruzy Madencilik A.Ş.</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] Ruzye 9.20₺ anlık ağır yükseldi, tradelik bakılır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>OZATD</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>OZATD</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Ozfatura Teknoloji A.Ş.</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>3120</v>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] 151 TL'den alınıp orta-uzun vade takip edilen analiz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>TEHOL</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>TEHOL</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Tek-Art Holding A.Ş.</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] %140.84 net kâr ile kapatılan analiz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>KCAER</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>KCAER</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Kocaer Çelik Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>15</v>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] Kcaer 11.14₺ tradelik değil değerlenme (%45).</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>DSTKF</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>DSTKF</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Destek Faktoring A.Ş.</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>2048</v>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>[Oğuz Analizi] Destek Faktoring tradelik takip (Giriş ~2.180 TL, Anlık ~2.048 TL).</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4477,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update Excel and tracking database with Ahmet Mergen live stream analysis
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H135"/>
+  <dimension ref="A1:H142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1504,12 +1504,20 @@
       <c r="D35" s="7" t="n">
         <v>17.63</v>
       </c>
-      <c r="E35" s="7" t="n"/>
-      <c r="F35" s="7" t="n"/>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>13.75 TL (50 Günlük HO)</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>22.52 TL</t>
+        </is>
+      </c>
       <c r="G35" s="7" t="n"/>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>[Oğuz Analizi] Mogan 12.75₺ buradan pozisyon açıyor (%60 prim).</t>
+          <t>[Ahmet Mergen] Eski alım yeri 7.50 TL'ydi. 22.52 TL büyük çanak tamamlanma direnci. Fiyat ortalamadan açıldığı için kâr satışı normal.</t>
         </is>
       </c>
     </row>
@@ -3805,15 +3813,23 @@
           <t>Tüpraş Türkiye Petrol Rafinerileri A.Ş.</t>
         </is>
       </c>
-      <c r="D113" s="7" t="n"/>
-      <c r="E113" s="7" t="n"/>
-      <c r="F113" s="8" t="n">
-        <v>340</v>
+      <c r="D113" s="7" t="n">
+        <v>292.25</v>
+      </c>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>275.00 - 280.00 TL</t>
+        </is>
+      </c>
+      <c r="F113" s="8" t="inlineStr">
+        <is>
+          <t>320.00 - 335.00 TL</t>
+        </is>
       </c>
       <c r="G113" s="7" t="n"/>
       <c r="H113" s="7" t="inlineStr">
         <is>
-          <t>[Ahmet Mergen Analizi] 50 haftalık ortalama destek. 6 dolar (kur hesabıyla 340-350 TL civarı) hedef ve direnç bölgesi.</t>
+          <t>[Ahmet Mergen] 4 haftada %50 yükseldi, tepede Doji oluştu. Petrol geri çekilmesiyle 275-280 TL 20 günlük HO desteğine süzülebilir. Çanak katlama hedefi 330-335 TL.</t>
         </is>
       </c>
     </row>
@@ -4441,6 +4457,251 @@
       <c r="H135" t="inlineStr">
         <is>
           <t>[Oğuz Analizi] Destek Faktoring tradelik takip (Giriş ~2.180 TL, Anlık ~2.048 TL).</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>USAK</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>USAK</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Uşak Seramik Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>1.34 - 1.35 TL</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>1.80 TL</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] 2024 ve 2025 eski dipleri 1.35-1.37 TL seviyesine geldi. Dolarda 2 cent dip seviyesi. Ortalamaların üzerine çıkması ve hacim beklenmeli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>YKBNK</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>YKBNK</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Yapı ve Kredi Bankası A.Ş.</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>32</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>28.00 - 30.00 TL (Dolarda 60 Cent)</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>36.00 TL</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Bankalarda 50 aylık ortalama test ediliyor. Dolarda 60 cent seviyesi kritik ana destek. 60 cent kırılırsa XBANK 2026 riski doğar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>PAHOL</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>PAHOL</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Pasifik Holding A.Ş.</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>1.25 - 1.32 TL</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>1.67 TL</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Yatay alandan aşağı sarkıyor. 1.32-1.35 ve 1.25 TL desteklerine süzülüyor. 50 günlük ortalama altında alım yönü zayıf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>SAHOL</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>SAHOL</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Sabancı Holding A.Ş.</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>85</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>75.00 - 80.00 TL</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>105.00 - 110.00 TL</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] 75-105 TL devasa yatay bant. 85 TL 4. dip bölgesi, esas ana toplama yeri 75 TL. 105 TL kırılırsa katlama hedefi 130-135 TL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>NUGYO</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>NUGYO</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Nurol GMYO A.Ş.</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>7.50 - 8.50 TL</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>12.00 - 14.00 TL</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Oynaklığı yüksek spekülatif tahta. 8.50 TL civarı alıcı bölgeleri. 12 TL üzerinde satıcı gelir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>NATEN</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>NATEN</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Natürel Yenilenebilir Enerji A.Ş.</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>6</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>5.00 - 5.50 TL</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>8.50 TL</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] 1.5 yıldır 50 haftalık ortalama altında düşüşte. Mumlar küçülüyor, 5.00-5.50 TL dip bölgesine yanaşma sinyali var.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>PETKM</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>PETKM</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Petkim Petrokimya A.Ş.</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>20</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>18.50 TL</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>23.50 TL</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Petrol sert yükselişiyle %50 primlendi, brent petrol düzeltmesiyle ortalamalara çekilme riski mevcut.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ASELS THYAO GARAN MGROS video analysis notes and tracking
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H142"/>
+  <dimension ref="A1:H146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -4702,6 +4702,104 @@
       <c r="H142" t="inlineStr">
         <is>
           <t>[Ahmet Mergen] Petrol sert yükselişiyle %50 primlendi, brent petrol düzeltmesiyle ortalamalara çekilme riski mevcut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>ASELS</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>ASELS</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Aselsan Elektronik Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>306.00 TL</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>340.00 TL</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>[Video Analizi] Savunma, yazılım ve teknoloji büyümesi güçlü; ancak çarpanları pahalı. 340, 320 ve 306 TL bölgeleri takip ediliyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>THYAO</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>THYAO</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Türk Hava Yolları A.O.</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>[Video Analizi] Yüksek döviz geliri ve uzun vadeli havacılık büyümesi olumlu; petrol fiyatları ve jeopolitik riskler olumsuz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>GARAN</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>GARAN</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Türkiye Garanti Bankası A.Ş.</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>[Video Analizi] Güçlü bankacılık altyapısı ve kurumsal sahiplik öne çıkıyor; fakat döviz geliri ve doğal kur koruması sınırlı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>MGROS</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>MGROS</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Migros Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>[Video Analizi] Gıda talebi krizlerde de sürer, nakit üretmesi ve online satış kanalları olumlu; kâr marjlarındaki gerileme risk.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add second Ahmet Mergen stream analyses (RYSAS TTRAK HALKB VAKBN PGSUS DOAS SISE)
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H146"/>
+  <dimension ref="A1:H153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -4800,6 +4800,251 @@
       <c r="H146" t="inlineStr">
         <is>
           <t>[Video Analizi] Gıda talebi krizlerde de sürer, nakit üretmesi ve online satış kanalları olumlu; kâr marjlarındaki gerileme risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>RYSAS</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>RYSAS</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Reysaş Taşımacılık ve Lojistik A.Ş.</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>24</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>21.64 TL (50 Günlük HO)</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>25.00 TL - 26.50 TL</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] 20 TL altından 24 TL'ye tepki verdi. 25.00 ve 26.50 TL ara dirençler. Çanak tamamlama potansiyeli mevcut. 50 günlük HO (21.64 TL) iz süren stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>TTRAK</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>TTRAK</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Türk Traktör ve Ziraat Makineleri A.Ş.</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>400</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>400.00 TL (Dolar: 5.5-6 USD)</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>500.00 TL (50 Günlük HO)</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] 1.000 TL'den 400 TL'ye süzüldü. %80'e yakın çekilme yaşandı. 500 TL (50 günlük HO) seviyesine %20'lik tepki hareketi yapabilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>HALKB</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>HALKB</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Türkiye Halk Bankası A.Ş.</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>29.00 - 30.00 TL (0.72 - 0.75 USD)</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>34.00 TL</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Dolar bazında 50 aylık ortalama (0.72-0.75$) dip bölgesine geldi. BIST bankacılık genel baskısı altında.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>VAKBN</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>VAKBN</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Türkiye Vakıflar Bankası T.A.O.</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>18.50 - 19.00 TL</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>22.00 TL</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] 50 aylık ortalama dip bölgesini test ediyor. Bankacılık dip kırılımları takibinde.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>PGSUS</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>PGSUS</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Pegasus Hava Taşımacılığı A.Ş.</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>154</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>135.00 - 150.00 TL</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>200.00 TL - 240.00 TL</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Petrol sıçraması ve jeopolitik riskle 285 TL'den 150 TL'ye (%50) sert geriledi. 135-150 TL dip bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>DOAS</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>DOAS</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Doğuş Otomotiv Servis ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>195</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>175.00 - 180.00 TL</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>210.00 TL</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Kısa vadede aşağı kayıyor. 175-180 TL yatay ana dip desteği. 195 TL üzerine çıkamazsa 180 TL'ye süzülebilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>SISE</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>SISE</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Türkiye Şişe ve Cam Fabrikaları A.Ş.</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>42</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>40.00 - 42.00 TL</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>48.00 TL</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] 42 TL seviyelerinde dip arayışında, baskı devam ediyor.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Eko TV Ahmet Mergen live stream analyses (SKBNK EUREN TMSN KCHOL ASELS, Crypto & Commodities)
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H153"/>
+  <dimension ref="A1:H157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -4721,19 +4721,22 @@
           <t>Aselsan Elektronik Sanayi A.Ş.</t>
         </is>
       </c>
+      <c r="D143" t="n">
+        <v>361.75</v>
+      </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>306.00 TL</t>
+          <t>300.00 - 320.00 TL (Ana Destek)</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>340.00 TL</t>
+          <t>388.00 TL - 406.00 TL</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>[Video Analizi] Savunma, yazılım ve teknoloji büyümesi güçlü; ancak çarpanları pahalı. 340, 320 ve 306 TL bölgeleri takip ediliyor.</t>
+          <t>[Ahmet Mergen Eko TV] Dikkatli olunmalı, stopsuz alım yapılmamalı. Geri çekilmelerde 300-320 TL ana alım/destek bölgesi.</t>
         </is>
       </c>
     </row>
@@ -5045,6 +5048,146 @@
       <c r="H153" t="inlineStr">
         <is>
           <t>[Ahmet Mergen] 42 TL seviyelerinde dip arayışında, baskı devam ediyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>SKBNK</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>SKBNK</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Şekerbank T.A.Ş.</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>5.00 - 6.00 TL</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>14.00 TL (Haftalık HO)</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen Eko TV] 20 TL'den 7.50 TL'ye düştü. Taban çözülme süreci takip edilmeli, 5.00-6.00 TL dip oluşum alanı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>EUREN</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>EUREN</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Europen Endüstri İnşaat Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>3.50 TL (Dolar: 0.08 USD Halka Arz Dibi)</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>4.50 - 5.00 TL (20 &amp; 50 Günlük HO)</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen Eko TV] Dolar bazında halka arz seviyesi olan 0.08 USD (8 cent) dibine geldi. 20 ve 50 günlük HO üzeri hareket takip edilmeli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>TMSN</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>TMSN</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Tümosan Motor ve Traktör Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>86</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>80.00 TL (Ana Taban)</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>89.00 TL (50G HO), 105.00 - 110.00 TL (Kanal)</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen Eko TV] 80 TL'den tepki verdi. Sağ omuz TOBO oluşumu var. 50 günlük HO (89 TL) aşılırsa kanal hedefi 105-110 TL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>KCHOL</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>KCHOL</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Koç Holding A.Ş.</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>190</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>185.00 TL (50 Haftalık HO) / 175.00 - 180.00 TL (%50 Fibo)</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>211.00 TL - 250.00 TL (Çanak Hedefi: 300+ TL)</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen Eko TV] 20 haftalık HO (193 TL) delindi. 50 haftalık HO (185 TL) ve 175-180 TL %50 Fibo ana destek bölgesi. Uzun vade hedef 300+ TL.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Emtia (Gold, Silver, Petrol, Copper) sensitivity correlation alerts and integrate Oğuz Telegram calls (AKFYE, PRKME, BETAE, NETCD, ENERY, TRALT)
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:H160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -531,6 +531,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -5188,6 +5189,81 @@
       <c r="H157" t="inlineStr">
         <is>
           <t>[Ahmet Mergen Eko TV] 20 haftalık HO (193 TL) delindi. 50 haftalık HO (185 TL) ve 175-180 TL %50 Fibo ana destek bölgesi. Uzun vade hedef 300+ TL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>AKFYE</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Akfen Yenilenebilir Enerji A.Ş.</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram] Buna 23₺'de 23,40₺ ortalama yapabilir. 24.50₺ direnç.</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>BETAE</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Beta Enerji ve Teknoloji A.Ş.</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>78</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram] Betae 78₺ tradelik bakılabilir.</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>TRALT</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Türk Altın İşletmeleri A.Ş.</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>12</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram / Emtia Takip] Altın emtiasına duyarlı altın madenciliği takibi.</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Integrate Oğuz Telegram Batch 3 calls (ZGYO, EKDMR, MEYSU, PENGD, PAHOL, KTLEV, PASEU, JANTS)
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -5262,6 +5262,106 @@
         </is>
       </c>
       <c r="G160" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>ZGYO</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Zergay Gayrimenkul Yatırım Ortaklığı A.Ş.</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram] Zgyo 33.90₺ takibe alındı.</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>PENGD</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Penguen Gıda Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram] Pengd 9,60₺ yine bakılabilir 9₺ dibi göz önünde tutularak.</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>KTLEV</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Katılımevim Tasarruf Finansman A.Ş.</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>37.28</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram] Ktlev alabilir (Tabandan %16 tepki).</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>JANTS</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Jantsa Jant Sanayi ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>14.85</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram] Jants 14,85₺ açılışta bakabiliriz 14,50₺ altı. 16₺ direnç.</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
         <is>
           <t>Oğuz</t>
         </is>

</xml_diff>

<commit_message>
Integrate Oğuz Telegram Batch 4 calls (ARFYE, INVEO, MIATK, EKDMR, YAYLA, NETCD, LOGO)
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H164"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -5362,6 +5362,56 @@
         </is>
       </c>
       <c r="G164" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>INVEO</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Inveo Yatırım Holding A.Ş.</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram] Inveo 6,98₺. Lakin 6,80 civarında stop olunabilir.</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>LOGO</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Logo Yazılım Sanayi ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>133.9</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram] Logo 133,90₺ buradan takip ediyorum (%5 kazanç).</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
         <is>
           <t>Oğuz</t>
         </is>

</xml_diff>

<commit_message>
Integrate Oğuz Telegram Batch 5 calls (ECOGR, SDTTR, FONET, ARFYE)
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H166"/>
+  <dimension ref="A1:H167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -5412,6 +5412,31 @@
         </is>
       </c>
       <c r="G166" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>ECOGR</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Ecogreen Enerji Holding A.Ş.</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram] Ecogr 34,40₺ trade verebilir.</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
         <is>
           <t>Oğuz</t>
         </is>

</xml_diff>

<commit_message>
Add ICUGS to Gold commodity correlation mapping and integrate Oğuz Telegram Batch 7 calls
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H167"/>
+  <dimension ref="A1:H168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -5437,6 +5437,31 @@
         </is>
       </c>
       <c r="G167" t="inlineStr">
+        <is>
+          <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>ICUGS</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>İşıklar Enerji ve Yapı Holding A.Ş.</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>[Oğuz Telegram / Altın Madenciliği] İcugs 5,42₺. Altın madenciliği faaliyetleri var, takibe alınabilir.</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
         <is>
           <t>Oğuz</t>
         </is>

</xml_diff>

<commit_message>
Expand Petrol commodity group (TUPRS, PETKM, TUKAS, FROTO, THYAO, PGSUS) and adjust Gold min_move threshold to 0.3% / Petrol to 0.4%
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H168"/>
+  <dimension ref="A1:H169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -5464,6 +5464,31 @@
       <c r="G168" t="inlineStr">
         <is>
           <t>Oğuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>TUKAS</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Tukaş Gıda Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Petrol / Akaryakıt lojistik ve tarım maliyeti takibi.</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Emtia / Petrol</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace TUKAS with TRCAS (Turcas Petrol) in Petrol commodity group
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H169"/>
+  <dimension ref="A1:H170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -5487,6 +5487,31 @@
         </is>
       </c>
       <c r="G169" t="inlineStr">
+        <is>
+          <t>Emtia / Petrol</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>TRCAS</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Turcas Petrol A.Ş.</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Petrol, Akaryakıt Dağıtım ve Enerji takibi.</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
         <is>
           <t>Emtia / Petrol</t>
         </is>

</xml_diff>

<commit_message>
Parse and integrate Ahmet Mergen YouTube transcript levels (ADES, CCOLA, AKBNK, BLCYT, NATEN) and update XU100 warning index logic
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H170"/>
+  <dimension ref="A1:H173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -613,18 +613,22 @@
           <t>AKBNK</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Akbank T.A.S.</t>
-        </is>
+      <c r="C5" s="7" t="n">
+        <v>67</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>62</v>
       </c>
       <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="9" t="n">
-        <v>24</v>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Akbank TOBO yapısında. 70 TL direnci aşılırsa 78-79 TL hedefi aktif olur. Stop 65.00-65.50 TL civarı konulmalı.</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Mergen</t>
+        </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
@@ -4647,10 +4651,8 @@
           <t>NATEN</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>Natürel Yenilenebilir Enerji A.Ş.</t>
-        </is>
+      <c r="C141" t="n">
+        <v>6</v>
       </c>
       <c r="D141" t="n">
         <v>6</v>
@@ -4662,7 +4664,12 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>8.50 TL</t>
+          <t>[Ahmet Mergen] Düşüş trendi sürüyor. Dolar bazlı 2022 dip seviyelerine (5.00-5.50 TL) süzülmüş durumda. Düşüşün durması için 50 haftalık HO üzerine geçilmeli.</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Mergen</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -5514,6 +5521,99 @@
       <c r="G170" t="inlineStr">
         <is>
           <t>Emtia / Petrol</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>ADES</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Adese Alışveriş Merkezleri Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D171" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E171" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Kağıt 80-85 kuruş civarında. Macera gibi bir şey olabilir. Spekülatif hareketle 1.20 TL ve 2.00-3.00 TL dirençleri hedeflenebilir.</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Mergen</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>CCOLA</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Coca-Cola İçecek A.Ş.</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>90</v>
+      </c>
+      <c r="D172" t="n">
+        <v>80</v>
+      </c>
+      <c r="E172" t="n">
+        <v>115</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Trend pozitif. 20 haftalık hareketli ortalama ve yükselen trend desteği kırılmadıkça vagonda kalmalı. 2.33-2.40 Dolar seviyeleri ana dirençtir.</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Mergen</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>BLCYT</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Bilici Yatırım Sanayi ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="D173" t="n">
+        <v>19</v>
+      </c>
+      <c r="E173" t="n">
+        <v>22</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen] Dolar bazlı tarihi dip seviyelerinde (2021 diplerine eşit). 22.00-23.70 TL geçilirse 29.00 TL çanak hedeflenebilir.</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Mergen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix live prices and redesign signal dashboard
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H173"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -531,7 +531,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -5614,6 +5613,457 @@
       <c r="G173" t="inlineStr">
         <is>
           <t>Mergen</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>mergen-20260811-xu100</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>XU100</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>BIST 100 Endeksi</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>13960</v>
+      </c>
+      <c r="F174" t="n">
+        <v>14254</v>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 13.958-13.960 üzeri hareket 14.250-14.254 direncini gündeme getirir. 14.254 kırılırsa 14.630, 14.876 ve 15.204; devamında 17.200-17.500 puanlık büyük çanak hedefi izlenebilir. Zaman: 00:00:13-00:04:32.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>mergen-20260811-yigit</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>YIGIT</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Yiğit Akü Malzemeleri Nakliyat Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>28</v>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 28-29 TL bölgesinde tıkanma var. Otomotiv sektörü zayıf olduğu için direnç aşılmadan güçlü hareket teyit edilmiş sayılmıyor. Zaman: 00:06:03-00:06:50.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>mergen-20260811-sasa</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>SASA</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Sasa Polyester Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>25</v>
+      </c>
+      <c r="E176" t="n">
+        <v>20.36</v>
+      </c>
+      <c r="F176" t="n">
+        <v>29</v>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 20,36-21,50 TL dip bölgesi. 20 TL altı zayıflama riski; 25 TL üzeri 29 TL'yi, 30 TL üzeri 39-40 TL eski tepe bölgesini gündeme getirir. Uzun vadeli ortalamaların altında olduğu için teyit beklenmeli. Zaman: 00:06:50-00:10:28 ve 00:32:50-00:37:19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>mergen-20260811-yayla</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>YAYLA</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Yayla Agro Gıda Sanayi ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>11</v>
+      </c>
+      <c r="E177" t="n">
+        <v>10</v>
+      </c>
+      <c r="F177" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 11 TL haftalık ortalama/teyit seviyesi. Birkaç kapanış 11 TL üzerinde kalırsa 12,50 ve 14-14,50 TL; devamında 15-16 TL potansiyeli değerlendirilebilir. Zaman: 00:11:45-00:14:23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>mergen-20260811-bobet</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>BOBET</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Boğaziçi Beton Sanayi ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>18</v>
+      </c>
+      <c r="E178" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F178" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 17,50-18 TL çoklu dip/tepki bölgesi. 16,50-16,75 TL altı stop düşünülebilir. 20,50-21 TL aşılırsa 24-24,20 TL; daha sonra 28,50-29 TL hedef/direnç bölgesi. Zaman: 00:14:56-00:19:52.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>mergen-20260811-cvkmd</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>CVKMD</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>CVK Maden İşletmeleri Sanayi ve Ticaret A.Ş.</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>15</v>
+      </c>
+      <c r="E179" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="F179" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 14,75-15 TL 20 haftalık ortalama/stop bölgesi; kırılırsa 12,50 TL 50 haftalık ortalama desteği izlenir. 18-18,50 TL sıkışma direnci aşılırsa 21,50-22 TL ve 25 TL hedefleri gündeme gelir. Zaman: 00:19:52-00:24:28.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>mergen-20260811-froto</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>FROTO</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Ford Otomotiv Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>62</v>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Endeks değişikliği kaynaklı yabancı fon satış baskısı vurgulandı. Mevcut dip bölgesi korunmazsa 62 TL derin destek/alım için yeniden değerlendirme seviyesi olarak belirtildi. Zaman: 00:25:21-00:32:50.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>mergen-20260811-halkb</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>HALKB</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Türkiye Halk Bankası A.Ş.</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Bedelli/sermaye işlemi belirsizliğiyle satış baskısı ve bankacılık endeksi desteğinin kritik olduğu belirtildi. İkili tepe senaryosundaki 40 cent hedef teknik ölçüm olarak anlatıldı, kesin beklenti olarak sunulmadı. Zaman: 00:37:19-00:40:35.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>mergen-20260811-xbank</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>XBANK</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>BIST Banka Endeksi</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Bankacılık endeksi uzun vadeli ortalama ve dip trend çizgisinde bıçak sırtında. Büyük bankalarda ortak satış sürerse genel endeks senaryosunun bozulacağı vurgulandı. Dolar bazlı 300-365 seviyeleri yorumlandığı için TL alarmı oluşturulmadı. Zaman: 00:39:37-00:42:23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>mergen-20260811-ulker</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>ULKER</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Ülker Bisküvi Sanayi A.Ş.</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>85</v>
+      </c>
+      <c r="E183" t="n">
+        <v>85</v>
+      </c>
+      <c r="F183" t="n">
+        <v>100</v>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Yaklaşık 85 TL/1,90 USD bölgesinde tarihsel diplerin altına sarkma var. BIST 14.250'yi büyük hisselerle geçmeden alım için acele edilmemesi; tepki halinde 100 TL ortalama bölgesinin izlenmesi söylendi. Zaman: 00:44:34-00:50:13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>mergen-20260811-naten</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>NATEN</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Natürel Yenilenebilir Enerji A.Ş.</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>5</v>
+      </c>
+      <c r="F184" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Dolar bazında 2022 diplerinin de altı ve yaklaşık 10 cent bölgesi. Çok düşmüş olsa da trend hâlâ negatif; 6,50 TL ve ardından 7,50 TL haftalık ortalamaları aşmadan teyit yok. Zaman: 00:50:13-00:53:02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>mergen-20260811-tavhl</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>TAVHL</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>TAV Havalimanları Holding A.Ş.</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>300</v>
+      </c>
+      <c r="E185" t="n">
+        <v>250</v>
+      </c>
+      <c r="F185" t="n">
+        <v>300</v>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Ana yatay bant 200-300 TL. 250 TL altı yeniden zayıflama, 215 TL derin destek; 300 TL üzerinde tutunma alıcı teyidi olarak değerlendirilebilir. Petrol yükselişi havacılık için risk. Zaman: 00:53:50-00:56:44.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>mergen-20260811-glrmk</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>GLRMK</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Gülermak Ağır Sanayi İnşaat ve Taahhüt A.Ş.</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>150</v>
+      </c>
+      <c r="F186" t="n">
+        <v>210</v>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 260 TL sonrası düşüşte 150-210 TL yatay bandı. Sağ omuz oluşumu tamamlanırsa TOBO ile yeniden 200 TL üzeri/210 TL tepe bölgesi gündeme gelebilir. Zaman: 01:07:25-01:08:58.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>mergen-20260811-brent</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>BZ=F</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Brent Petrol ($)</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>80</v>
+      </c>
+      <c r="F187" t="n">
+        <v>90.75</v>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 90,61-90,75 dolar boşluk/ilk direnç. 95-96 dolar enflasyon ve faiz riski; 98 dolar kırılırsa 115-116 dolar teknik hedef senaryosu. 80 dolar altı yeniden zayıflama. Zaman: 00:59:38-01:03:23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>mergen-20260811-gold</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>GC=F</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Ons Altın ($)</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>4200</v>
+      </c>
+      <c r="F188" t="n">
+        <v>4600</v>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 4.382 dolar civarı kâr alma bölgesi olarak değerlendirildi. 4.000-4.200 dolar ortalama/destek alanı; trend korunursa 4.600 dolar civarında yeniden satıcı bekleniyor. Petrol 95-96 dolara giderse 4.200'e düzeltme riski. Zaman: 01:03:23-01:05:01.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>mergen-20260811-silver</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>SI=F</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Ons Gümüş ($)</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>65</v>
+      </c>
+      <c r="E189" t="n">
+        <v>64</v>
+      </c>
+      <c r="F189" t="n">
+        <v>71</v>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 64-65 dolar kırılımı ve yaklaşan golden cross pozitif. Teknik hedef/direnç 71 dolar; hızlı yükseliş sonrasında düzeltme riskine karşı stoplu izlenmeli. Zaman: 01:05:01-01:07:25.</t>
         </is>
       </c>
     </row>
@@ -5631,7 +6081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G209"/>
+  <dimension ref="A1:G251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12897,6 +13347,1476 @@
         </is>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>XU100</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>BIST 100 Endeksi</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>13960</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 13.960 üzeri 14.250-14.254 hareketi tetiklenebilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>XU100</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>BIST 100 Endeksi</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>14254</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Ana direnç kırılımı; 14.630 ve 14.876 hedefleri izlenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>XU100</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>BIST 100 Endeksi</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>14630</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] İlk üst hedef görüldü.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>XU100</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>BIST 100 Endeksi</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>14876</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] İkinci üst hedef görüldü.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>XU100</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>BIST 100 Endeksi</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>15204</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] TOBO/çanak hedef bölgesi görüldü.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>YIGIT.IS</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Yiğit Akü</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>28</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 28-29 TL direnç bölgesine geldi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>SASA.IS</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Sasa Polyester</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>20</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 20 TL altı zayıflama riski.</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>SASA.IS</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Sasa Polyester</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>25</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 25 TL üzeri 29 TL potansiyeli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>SASA.IS</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Sasa Polyester</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>29</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 29 TL yatay bant direnci.</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>SASA.IS</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Sasa Polyester</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>30</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 30 TL üzeri 39-40 TL eski tepe senaryosu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>YAYLA.IS</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Yayla Agro Gıda</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>11</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Haftalık ortalama/teyit seviyesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>YAYLA.IS</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Yayla Agro Gıda</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] İlk hedef görüldü; 14-14,50 izlenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>YAYLA.IS</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Yayla Agro Gıda</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] İkinci hedef/direnç görüldü.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>BOBET.IS</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Boğaziçi Beton</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>18</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 17,50-18 TL çoklu dip/tepki bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>BOBET.IS</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Boğaziçi Beton</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>16.75</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Analistin belirttiği stop bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>BOBET.IS</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Boğaziçi Beton</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 20,50-21 TL ilk direnç.</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>BOBET.IS</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Boğaziçi Beton</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>24</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 24-24,20 TL hedef/direnç.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>BOBET.IS</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Boğaziçi Beton</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 28,50-29 TL üst hedef.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>CVKMD.IS</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>CVK Maden</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 20 haftalık ortalama/stop bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>CVKMD.IS</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>CVK Maden</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 50 haftalık ortalama desteği.</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>CVKMD.IS</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>CVK Maden</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Sıkışma direnci; kırılımda 21,50-22 ve 25 hedefleri.</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>CVKMD.IS</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>CVK Maden</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] İlk üst hedef bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>CVKMD.IS</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>CVK Maden</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>25</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Ana teknik hedef.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>FROTO.IS</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Ford Otosan</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>62</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Derin destek/yeniden değerlendirme seviyesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>ULKER.IS</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Ülker Bisküvi</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>85</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Tarihsel dip bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>ULKER.IS</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Ülker Bisküvi</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>100</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Tepki hedefi/ortalama bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>NATEN.IS</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Natürel Enerji</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>5</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Aşırı düşüş/dip bölgesi; trend teyidi yok.</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>NATEN.IS</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Natürel Enerji</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] İlk haftalık ortalama/teyit seviyesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>NATEN.IS</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Natürel Enerji</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] İkinci haftalık ortalama/teyit seviyesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>TAVHL.IS</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>TAV Havalimanları</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>250</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 250 TL altı zayıflama.</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>TAVHL.IS</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>TAV Havalimanları</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>215</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Derin destek bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>TAVHL.IS</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>TAV Havalimanları</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>300</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 300 TL üzerinde tutunma alıcı teyidi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>GLRMK.IS</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Gülermak Ağır Sanayi</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>150</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 150-210 TL yatay bandın alt sınırı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>GLRMK.IS</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Gülermak Ağır Sanayi</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>210</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] TOBO ihtimalinde tepe/direnç bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>BZ=F</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Brent Petrol</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>80</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 80 dolar altı zayıflama.</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>BZ=F</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Brent Petrol</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>90.75</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 90,61-90,75 dolar boşluk/direnç bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>BZ=F</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Brent Petrol</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>96</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Enflasyon ve faiz riski artan kritik bölge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>BZ=F</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Brent Petrol</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>98</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Kırılımda 115-116 dolar teknik hedef senaryosu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>GC=F</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Ons Altın</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>4200</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Ortalama/destek ve trend kontrol bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>GC=F</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Ons Altın</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>4600</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Kâr satışı beklenen hedef/direnç bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>SI=F</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Ons Gümüş</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>65</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 64-65 dolar kırılım teyidi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>SI=F</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Ons Gümüş</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>71</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Teknik hedef/direnç bölgesi.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
add conditional analyst levels from Mergen video
</commit_message>
<xml_diff>
--- a/Hisselerin_Teknik_Verileri.xlsx
+++ b/Hisselerin_Teknik_Verileri.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -6067,6 +6067,68 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>mergen-20260811-taten</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>TATEN</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Tatlıpınar Enerji Üretim A.Ş.</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="E190" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F190" t="n">
+        <v>21</v>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 6,50-7,00 TL geçmiş dip/tepki bölgesi olarak izleniyor; mali görünüm zayıf olduğu için yalnızca destek üzerinde tutunma ve en az 1-2 hafta teyit sonrası değerlendirme yapılmalı. 21 TL güçlü satış/direnç bölgesi. 5 TL video seviyesi değildir; 5 TL'ye sarkma 6,50-7,00 desteğinin kırıldığı risk senaryosudur. Zaman: 00:22:47-00:24:35.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>mergen-20260811-thyao</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>THYAO</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Türk Hava Yolları A.O.</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>315</v>
+      </c>
+      <c r="E191" t="n">
+        <v>310</v>
+      </c>
+      <c r="F191" t="n">
+        <v>325</v>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 315 TL üzeri toparlanma 325 TL'yi; formasyon teyidiyle yaklaşık 355 TL hedefini gündeme getirir. 310 TL altı kısa vadeli stop/bozulma seviyesi olarak takip edilmeli. Zaman: 00:15:39-00:18:55.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -6081,7 +6143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G251"/>
+  <dimension ref="A1:G257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -14817,6 +14879,216 @@
         </is>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>TATEN.IS</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Tatlıpınar Enerji</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 6,50-7 TL geçmiş dip/tepki bölgesi; mali teyit olmadan alım sinyali değildir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>TATEN.IS</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Tatlıpınar Enerji</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>5</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 6,50-7 TL desteği kırılmış olur; tepki garantisi değil, yüksek risk/izleme alarmı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>TATEN.IS</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Tatlıpınar Enerji</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>21</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Güçlü satış/direnç bölgesi; kâr realizasyonu değerlendirilebilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>THYAO.IS</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Türk Hava Yolları</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>315</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] 315 TL üzeri toparlanma teyidi; 325 TL izlenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>THYAO.IS</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Türk Hava Yolları</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Fiyat &lt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>310</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Kısa vadeli stop/bozulma seviyesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>THYAO.IS</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Türk Hava Yolları</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Fiyat &gt;= Hedef</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>355</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Evet</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Bekliyor</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>[Ahmet Mergen][2026-08-11 Transcript] Formasyon hedef bölgesi.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>